<commit_message>
Fix: Corrected winning number regex and news store limit in auto_update.py
</commit_message>
<xml_diff>
--- a/geocoded_cache_healthy.xlsx
+++ b/geocoded_cache_healthy.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -550,6 +550,163 @@
         <v>127.112688386546</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>수동 
+1등</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>37.7427114349339</v>
+      </c>
+      <c r="C11" t="n">
+        <v>127.296206187177</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>부산 금정구</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>35.2427772019609</v>
+      </c>
+      <c r="C12" t="n">
+        <v>129.092095292484</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>광주 서구</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>35.1520722691295</v>
+      </c>
+      <c r="C13" t="n">
+        <v>126.890187526298</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>울산 동구</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>35.5046358750559</v>
+      </c>
+      <c r="C14" t="n">
+        <v>129.416487775873</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>경기 화성시</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>37.1995372034717</v>
+      </c>
+      <c r="C15" t="n">
+        <v>126.831477350333</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>경기 포천시</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>37.8949928340087</v>
+      </c>
+      <c r="C16" t="n">
+        <v>127.200332890652</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>경기 시흥시</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>37.3801150715958</v>
+      </c>
+      <c r="C17" t="n">
+        <v>126.802977796436</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>경남 김해시</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>35.228565355864</v>
+      </c>
+      <c r="C18" t="n">
+        <v>128.88936269803</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>경북 고령군</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>35.7260653208402</v>
+      </c>
+      <c r="C19" t="n">
+        <v>128.262895757558</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>제주 서귀포시</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>33.2540646255023</v>
+      </c>
+      <c r="C20" t="n">
+        <v>126.559563466911</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>전남 영암군</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>34.8000591144732</v>
+      </c>
+      <c r="C21" t="n">
+        <v>126.696762590551</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>강원 춘천시</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>37.8812440340087</v>
+      </c>
+      <c r="C22" t="n">
+        <v>127.730207024668</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>